<commit_message>
ran a bunch of experiments
</commit_message>
<xml_diff>
--- a/wrapping_data/exel/model_results_first_better_try.xlsx
+++ b/wrapping_data/exel/model_results_first_better_try.xlsx
@@ -8,8 +8,11 @@
   </bookViews>
   <sheets>
     <sheet name="Model_Info" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="hidden_dim_32" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="hidden_dim_64" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="hidden_dim_16" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="hidden_dim_32" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="hidden_dim_64" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="hidden_dim_128" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="hidden_dim_256" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -529,35 +532,67 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>NodeOCGIN</t>
-        </is>
-      </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
           <t>NodeOCGIN</t>
         </is>
       </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>NodeOCGIN</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>NodeOCGIN</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>NodeOCGIN</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>num_layers</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C2" t="n">
         <v>3</v>
       </c>
-      <c r="B2" t="n">
+      <c r="D2" t="n">
+        <v>4</v>
+      </c>
+      <c r="E2" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
-        <v>0.2409390444810544</v>
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>test_rate</t>
+        </is>
       </c>
       <c r="B3" t="n">
-        <v>0.2088138385502471</v>
+        <v>0.1305601317957166</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.1297364085667216</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.07701812191103789</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.17833607907743</v>
       </c>
     </row>
     <row r="6">
@@ -574,74 +609,178 @@
         </is>
       </c>
       <c r="B7" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="C7" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C7" s="1" t="n">
+      <c r="D7" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="E7" s="1" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>0.01</v>
+        <v>0.001</v>
       </c>
       <c r="B8" t="n">
-        <v>0.1556836902800659</v>
+        <v>0.3966227347611203</v>
       </c>
       <c r="C8" t="n">
-        <v>0.200164744645799</v>
+        <v>0.164332784184514</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.1062602965403624</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.2178747940691927</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>0.03</v>
+        <v>0.005</v>
       </c>
       <c r="B9" t="n">
-        <v>0.2191103789126853</v>
+        <v>0.357495881383855</v>
       </c>
       <c r="C9" t="n">
-        <v>0.1952224052718287</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+        <v>0.228995057660626</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.1169686985172982</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.1449752883031301</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="B10" t="n">
+        <v>0.4497528830313015</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0.1717462932454695</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.1190280065897858</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.1548599670510708</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="B11" t="n">
+        <v>0.1857495881383855</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0.1289126853377265</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.1688632619439868</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.107495881383855</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>Model: NodeOCGINLossConstrains, Constrains: constrains/data/Cora_auto_generated_3_101_102_103.json</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="1" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
         <is>
           <t>l_factor</t>
         </is>
       </c>
-      <c r="B13" s="1" t="n">
+      <c r="B15" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="C15" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C13" s="1" t="n">
+      <c r="D15" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="E15" s="1" t="n">
         <v>5</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="1" t="n">
+    <row r="16">
+      <c r="A16" s="1" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="B16" t="n">
+        <v>0.3826194398682043</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0.1985172981878089</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.2104612850082372</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.1544481054365733</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="B17" t="n">
+        <v>0.2265238879736409</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0.1700988467874794</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0.120675453047776</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0.2380560131795717</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="n">
         <v>0.01</v>
       </c>
-      <c r="B14" t="n">
-        <v>0.2030477759472817</v>
-      </c>
-      <c r="C14" t="n">
-        <v>0.250823723228995</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="1" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="B15" t="n">
-        <v>0.1771004942339374</v>
-      </c>
-      <c r="C15" t="n">
-        <v>0.2586490939044481</v>
+      <c r="B18" t="n">
+        <v>0.2462932454695222</v>
+      </c>
+      <c r="C18" t="n">
+        <v>0.2285831960461285</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0.2162273476112026</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0.06836902800658978</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="B19" t="n">
+        <v>0.4373970345963756</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0.2051070840197693</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0.2240527182866557</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0.1602141680395387</v>
       </c>
     </row>
   </sheetData>
@@ -655,35 +794,67 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>NodeOCGIN</t>
-        </is>
-      </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
           <t>NodeOCGIN</t>
         </is>
       </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>NodeOCGIN</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>NodeOCGIN</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>NodeOCGIN</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>num_layers</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C2" t="n">
         <v>3</v>
       </c>
-      <c r="B2" t="n">
+      <c r="D2" t="n">
+        <v>4</v>
+      </c>
+      <c r="E2" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
-        <v>0.221169686985173</v>
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>test_rate</t>
+        </is>
       </c>
       <c r="B3" t="n">
-        <v>0.2763591433278418</v>
+        <v>0.2644151565074135</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.1692751235584843</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.1511532125205931</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.2454695222405272</v>
       </c>
     </row>
     <row r="6">
@@ -700,74 +871,964 @@
         </is>
       </c>
       <c r="B7" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="C7" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C7" s="1" t="n">
+      <c r="D7" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="E7" s="1" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>0.01</v>
+        <v>0.001</v>
       </c>
       <c r="B8" t="n">
-        <v>0.199341021416804</v>
+        <v>0.3937397034596375</v>
       </c>
       <c r="C8" t="n">
-        <v>0.3051894563426689</v>
+        <v>0.2092257001647446</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.2261120263591433</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.1820428336079077</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>0.03</v>
+        <v>0.005</v>
       </c>
       <c r="B9" t="n">
-        <v>0.1519769357495881</v>
+        <v>0.4703459637561779</v>
       </c>
       <c r="C9" t="n">
-        <v>0.2512355848434926</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+        <v>0.1149093904448105</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.2742998352553542</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.2495881383855025</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="B10" t="n">
+        <v>0.3537891268533773</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0.2948929159802307</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.228171334431631</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.2689456342668863</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="B11" t="n">
+        <v>0.0943163097199341</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0.1820428336079077</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.1902800658978583</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.2380560131795717</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>Model: NodeOCGINLossConstrains, Constrains: constrains/data/Cora_auto_generated_3_101_102_103.json</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="1" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
         <is>
           <t>l_factor</t>
         </is>
       </c>
-      <c r="B13" s="1" t="n">
+      <c r="B15" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="C15" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C13" s="1" t="n">
+      <c r="D15" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="E15" s="1" t="n">
         <v>5</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="1" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="B16" t="n">
+        <v>0.2961285008237232</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0.1515650741350906</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.292833607907743</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.2174629324546952</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="B17" t="n">
+        <v>0.278006589785832</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0.2590609555189456</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0.1919275123558484</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0.1684514003294893</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="B18" t="n">
+        <v>0.5395387149917628</v>
+      </c>
+      <c r="C18" t="n">
+        <v>0.2063426688632619</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0.2104612850082372</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0.2232289950576606</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="B19" t="n">
+        <v>0.3850906095551895</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0.2475288303130148</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0.2248764415156508</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0.2462932454695222</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>NodeOCGIN</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>NodeOCGIN</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>NodeOCGIN</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>NodeOCGIN</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>num_layers</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D2" t="n">
+        <v>4</v>
+      </c>
+      <c r="E2" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>test_rate</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0.306836902800659</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.2660626029654036</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.2635914332784184</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.2775947281713344</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Model: NodeOCGINLossConstrains, Constrains: constrains/data/Cora_auto_generated_2_101_102_103.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>l_factor</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="C7" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="D7" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="E7" s="1" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="B8" t="n">
+        <v>0.4184514003294893</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0.2347611202635914</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.2240527182866557</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.2116968698517298</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="B9" t="n">
+        <v>0.3912685337726524</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0.2458813838550247</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.2331136738056013</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.2784184514003295</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="B10" t="n">
+        <v>0.264003294892916</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0.2565897858319605</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.2961285008237232</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.242998352553542</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="B11" t="n">
+        <v>0.3595551894563427</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0.09390444810543658</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.2557660626029654</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.2549423393739704</v>
+      </c>
+    </row>
     <row r="14">
-      <c r="A14" s="1" t="n">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Model: NodeOCGINLossConstrains, Constrains: constrains/data/Cora_auto_generated_3_101_102_103.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>l_factor</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="C15" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="D15" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="E15" s="1" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="B16" t="n">
+        <v>0.3953871499176277</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0.2516474464579901</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.3830313014827018</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.2734761120263591</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="B17" t="n">
+        <v>0.2574135090609555</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0.2174629324546952</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0.3204283360790774</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0.3002471169686985</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="n">
         <v>0.01</v>
       </c>
-      <c r="B14" t="n">
-        <v>0.2088138385502471</v>
-      </c>
-      <c r="C14" t="n">
-        <v>0.2911861614497529</v>
+      <c r="B18" t="n">
+        <v>0.3422570016474464</v>
+      </c>
+      <c r="C18" t="n">
+        <v>0.35667215815486</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0.2483525535420099</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0.1960461285008237</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="B19" t="n">
+        <v>0.3801482701812191</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0.2887149917627677</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0.3241350906095552</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0.2228171334431631</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>NodeOCGIN</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>NodeOCGIN</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>NodeOCGIN</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>NodeOCGIN</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>num_layers</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D2" t="n">
+        <v>4</v>
+      </c>
+      <c r="E2" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>test_rate</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0.3336079077429984</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.1799835255354201</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.2397034596375618</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.221993410214168</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Model: NodeOCGINLossConstrains, Constrains: constrains/data/Cora_auto_generated_2_101_102_103.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>l_factor</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="C7" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="D7" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="E7" s="1" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="B8" t="n">
+        <v>0.2541186161449753</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0.2532948929159802</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.3014827018121911</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.2557660626029654</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="B9" t="n">
+        <v>0.3352553542009885</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0.2240527182866557</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.2631795716639209</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.2145799011532125</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="B10" t="n">
+        <v>0.2862438220757825</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0.2479406919275124</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.320840197693575</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.2755354200988468</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="B11" t="n">
+        <v>0.3364909390444811</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0.2079901153212521</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.2821252059308073</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.257001647446458</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Model: NodeOCGINLossConstrains, Constrains: constrains/data/Cora_auto_generated_3_101_102_103.json</t>
+        </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="B15" t="n">
-        <v>0.2598846787479407</v>
-      </c>
-      <c r="C15" t="n">
-        <v>0.2261120263591433</v>
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>l_factor</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="C15" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="D15" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="E15" s="1" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="B16" t="n">
+        <v>0.2405271828665568</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0.2524711696869852</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.2602965403624382</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.2458813838550247</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="B17" t="n">
+        <v>0.3492586490939045</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0.2397034596375618</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0.2343492586490939</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0.2841845140032949</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="B18" t="n">
+        <v>0.3657331136738056</v>
+      </c>
+      <c r="C18" t="n">
+        <v>0.2199341021416804</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0.2343492586490939</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0.2331136738056013</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="B19" t="n">
+        <v>0.2734761120263591</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0.221169686985173</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0.2759472817133443</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0.2841845140032949</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>NodeOCGIN</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>NodeOCGIN</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>NodeOCGIN</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>NodeOCGIN</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>num_layers</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D2" t="n">
+        <v>4</v>
+      </c>
+      <c r="E2" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>test_rate</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0.3261943986820428</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.03047775947281713</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.1046128500823723</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.02924217462932455</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Model: NodeOCGINLossConstrains, Constrains: constrains/data/Cora_auto_generated_2_101_102_103.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>l_factor</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="C7" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="D7" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="E7" s="1" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="B8" t="n">
+        <v>0.3480230642504119</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0.171334431630972</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.2314662273476112</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.03336079077429983</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="B9" t="n">
+        <v>0.2022240527182867</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0.1688632619439868</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.2557660626029654</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.2537067545304778</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="B10" t="n">
+        <v>0.1857495881383855</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0.1651565074135091</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.1499176276771005</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.2248764415156508</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="B11" t="n">
+        <v>0.3088962108731466</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0.2178747940691927</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.2405271828665568</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.02924217462932455</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Model: NodeOCGINLossConstrains, Constrains: constrains/data/Cora_auto_generated_3_101_102_103.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>l_factor</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="C15" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="D15" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="E15" s="1" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="B16" t="n">
+        <v>0.3467874794069193</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0.2026359143327842</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.2767710049423394</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.2162273476112026</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="B17" t="n">
+        <v>0.3056013179571664</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0.2343492586490939</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0.2046952224052718</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0.1598023064250412</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="B18" t="n">
+        <v>0.3233113673805602</v>
+      </c>
+      <c r="C18" t="n">
+        <v>0.149505766062603</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0.17833607907743</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0.1956342668863262</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="B19" t="n">
+        <v>0.2878912685337727</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0.221993410214168</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0.2327018121911038</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0.09761120263591433</v>
       </c>
     </row>
   </sheetData>

</xml_diff>